<commit_message>
Day 2: sort, filter, orders analysis
</commit_message>
<xml_diff>
--- a/excel/budget_practice.xlsx
+++ b/excel/budget_practice.xlsx
@@ -128,7 +128,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="171" formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -286,15 +286,15 @@
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -303,6 +303,144 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+        <horizontal style="thin">
+          <color auto="1"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+        <horizontal style="thin">
+          <color auto="1"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+        <horizontal style="thin">
+          <color auto="1"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+        <horizontal style="thin">
+          <color auto="1"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+        <horizontal style="thin">
+          <color auto="1"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -337,144 +475,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-        <horizontal style="thin">
-          <color auto="1"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="171" formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-        <horizontal style="thin">
-          <color auto="1"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-        <horizontal style="thin">
-          <color auto="1"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-        <horizontal style="thin">
-          <color auto="1"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-        <horizontal style="thin">
-          <color auto="1"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -489,7 +489,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F0D79DC-F8CB-4E29-9A05-A1D9D4DED54E}" name="Table1" displayName="Table1" ref="A1:E16" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="7" tableBorderDxfId="8" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F0D79DC-F8CB-4E29-9A05-A1D9D4DED54E}" name="Table1" displayName="Table1" ref="A1:E16" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
   <autoFilter ref="A1:E16" xr:uid="{9F0D79DC-F8CB-4E29-9A05-A1D9D4DED54E}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -498,11 +498,11 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{1CE644FE-3313-460B-A14A-17C7016A2457}" name="Date" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{E9203F67-D879-4EDA-9E0E-512377A50616}" name="Category" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{C8236E92-3C41-418A-ABDB-DFBDFD6C02A3}" name="Description" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{502423D8-1BFF-418A-94E1-F1A2612FE8DF}" name="Amount" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{3322DF51-E22F-49D5-B763-B8B6E9F038B1}" name="Payment method" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{1CE644FE-3313-460B-A14A-17C7016A2457}" name="Date" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{E9203F67-D879-4EDA-9E0E-512377A50616}" name="Category" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{C8236E92-3C41-418A-ABDB-DFBDFD6C02A3}" name="Description" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{502423D8-1BFF-418A-94E1-F1A2612FE8DF}" name="Amount" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{3322DF51-E22F-49D5-B763-B8B6E9F038B1}" name="Payment method" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Day 3: IF formulas, delay analysis
</commit_message>
<xml_diff>
--- a/excel/budget_practice.xlsx
+++ b/excel/budget_practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnuRavindra\Documents\GitHub\data-analyst-capstone\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9404BA69-09BB-41D7-9310-2B80D5C4BC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7CF29E-1945-4899-9506-75A0492D2537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E7F0E920-1D0C-48ED-90F0-15FD72CF6CA2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="34">
   <si>
     <t>Date</t>
   </si>
@@ -121,6 +121,12 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>Column2</t>
   </si>
 </sst>
 </file>
@@ -130,7 +136,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +148,12 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -302,7 +314,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="11">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -419,23 +437,23 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
+      <border>
         <bottom style="thin">
           <color auto="1"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
         <bottom style="thin">
           <color auto="1"/>
         </bottom>
@@ -489,20 +507,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F0D79DC-F8CB-4E29-9A05-A1D9D4DED54E}" name="Table1" displayName="Table1" ref="A1:E16" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
-  <autoFilter ref="A1:E16" xr:uid="{9F0D79DC-F8CB-4E29-9A05-A1D9D4DED54E}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F0D79DC-F8CB-4E29-9A05-A1D9D4DED54E}" name="Table1" displayName="Table1" ref="A1:G16" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:G16" xr:uid="{9F0D79DC-F8CB-4E29-9A05-A1D9D4DED54E}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
     <filterColumn colId="3" hiddenButton="1"/>
     <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{1CE644FE-3313-460B-A14A-17C7016A2457}" name="Date" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{E9203F67-D879-4EDA-9E0E-512377A50616}" name="Category" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{C8236E92-3C41-418A-ABDB-DFBDFD6C02A3}" name="Description" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{502423D8-1BFF-418A-94E1-F1A2612FE8DF}" name="Amount" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{3322DF51-E22F-49D5-B763-B8B6E9F038B1}" name="Payment method" dataDxfId="0"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{1CE644FE-3313-460B-A14A-17C7016A2457}" name="Date" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{E9203F67-D879-4EDA-9E0E-512377A50616}" name="Category" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{C8236E92-3C41-418A-ABDB-DFBDFD6C02A3}" name="Description" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{502423D8-1BFF-418A-94E1-F1A2612FE8DF}" name="Amount" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{3322DF51-E22F-49D5-B763-B8B6E9F038B1}" name="Payment method" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{141289AA-D09E-4A69-B2DF-E24F43E050BF}" name="Column1" dataDxfId="1">
+      <calculatedColumnFormula>IF(D2&gt;500,"Big","Small")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{0D5ECD5F-A026-478E-A988-BE002C5661C3}" name="Column2" dataDxfId="0">
+      <calculatedColumnFormula>IF(AND(B2="Food", D2&gt;500), "Watch", "Fine")</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -805,7 +831,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1D9A10D-F87D-4492-8A00-D4ED6F9A53BE}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -815,7 +841,7 @@
     <col min="5" max="5" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -831,8 +857,14 @@
       <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>46300</v>
       </c>
@@ -848,8 +880,16 @@
       <c r="E2" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2" t="str">
+        <f t="shared" ref="F2:F16" si="0">IF(D2&gt;500,"Big","Small")</f>
+        <v>Big</v>
+      </c>
+      <c r="G2" t="str">
+        <f t="shared" ref="G2:G16" si="1">IF(AND(B2="Food", D2&gt;500), "Watch", "Fine")</f>
+        <v>Watch</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>46301</v>
       </c>
@@ -865,8 +905,16 @@
       <c r="E3" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G3" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>46302</v>
       </c>
@@ -882,8 +930,16 @@
       <c r="E4" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>46303</v>
       </c>
@@ -899,8 +955,16 @@
       <c r="E5" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>46304</v>
       </c>
@@ -916,8 +980,16 @@
       <c r="E6" s="6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F6" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>46305</v>
       </c>
@@ -933,8 +1005,16 @@
       <c r="E7" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F7" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>46306</v>
       </c>
@@ -950,8 +1030,16 @@
       <c r="E8" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>Big</v>
+      </c>
+      <c r="G8" t="str">
+        <f t="shared" si="1"/>
+        <v>Watch</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>46307</v>
       </c>
@@ -967,8 +1055,16 @@
       <c r="E9" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G9" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>46308</v>
       </c>
@@ -984,8 +1080,16 @@
       <c r="E10" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>46309</v>
       </c>
@@ -1001,8 +1105,16 @@
       <c r="E11" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>Big</v>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>46310</v>
       </c>
@@ -1018,8 +1130,16 @@
       <c r="E12" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F12" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G12" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>46311</v>
       </c>
@@ -1035,8 +1155,16 @@
       <c r="E13" s="6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F13" t="str">
+        <f t="shared" si="0"/>
+        <v>Big</v>
+      </c>
+      <c r="G13" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>46312</v>
       </c>
@@ -1052,8 +1180,16 @@
       <c r="E14" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F14" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G14" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>46313</v>
       </c>
@@ -1069,8 +1205,16 @@
       <c r="E15" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F15" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G15" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="7">
         <v>46314</v>
       </c>
@@ -1085,6 +1229,14 @@
       </c>
       <c r="E16" s="2" t="s">
         <v>11</v>
+      </c>
+      <c r="F16" t="str">
+        <f t="shared" si="0"/>
+        <v>Small</v>
+      </c>
+      <c r="G16" t="str">
+        <f t="shared" si="1"/>
+        <v>Fine</v>
       </c>
     </row>
     <row r="18" spans="3:4" x14ac:dyDescent="0.35">
@@ -1097,6 +1249,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>